<commit_message>
housekeeping, add gif for readme
also, set up for scenario 1, a long, flow only simulation for continuous display/looping and scenario 2, a shorter demo of contaminant transport from well 2 to well 6 in the confined aquifer.
</commit_message>
<xml_diff>
--- a/layered_groundwater_model/inputs/scenarios_short3.xlsx
+++ b/layered_groundwater_model/inputs/scenarios_short3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krasows2\Documents\GitHub\isws-demonstration-models\layered_groundwater_model\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8B1586-1297-45C8-B902-478D20E80FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0208D788-05A3-4BBC-8F5E-535258C9B39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA5C4861-9FAE-4E22-824A-E10008A1D0F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{FA5C4861-9FAE-4E22-824A-E10008A1D0F9}"/>
   </bookViews>
   <sheets>
     <sheet name="s1" sheetId="1" r:id="rId1"/>
@@ -554,7 +554,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -20125,7 +20125,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E97801-BE61-4957-84E2-2B0DE4A8E880}">
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
@@ -20195,7 +20195,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -20272,7 +20272,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -20337,7 +20337,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -20402,7 +20402,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -20467,7 +20467,7 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -20532,7 +20532,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -20597,7 +20597,7 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -20662,7 +20662,7 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -20727,7 +20727,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -20792,7 +20792,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -20857,7 +20857,7 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -20949,7 +20949,7 @@
         <v>0</v>
       </c>
       <c r="N13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13">
         <v>0</v>
@@ -21014,7 +21014,7 @@
         <v>0</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14">
         <v>0</v>
@@ -21079,7 +21079,7 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -21117,7 +21117,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -21182,7 +21182,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -24155,6 +24155,3906 @@
         <v>0</v>
       </c>
       <c r="U62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>60</v>
+      </c>
+      <c r="B63">
+        <v>61</v>
+      </c>
+      <c r="C63" t="b">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>0</v>
+      </c>
+      <c r="J63">
+        <v>0</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+      <c r="L63">
+        <v>0</v>
+      </c>
+      <c r="M63">
+        <v>0</v>
+      </c>
+      <c r="N63">
+        <v>0</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>0</v>
+      </c>
+      <c r="Q63">
+        <v>0</v>
+      </c>
+      <c r="R63">
+        <v>0</v>
+      </c>
+      <c r="S63">
+        <v>0</v>
+      </c>
+      <c r="T63">
+        <v>0</v>
+      </c>
+      <c r="U63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>61</v>
+      </c>
+      <c r="B64">
+        <v>62</v>
+      </c>
+      <c r="C64" t="b">
+        <v>0</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+      <c r="L64">
+        <v>0</v>
+      </c>
+      <c r="M64">
+        <v>0</v>
+      </c>
+      <c r="N64">
+        <v>0</v>
+      </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64">
+        <v>0</v>
+      </c>
+      <c r="Q64">
+        <v>0</v>
+      </c>
+      <c r="R64">
+        <v>0</v>
+      </c>
+      <c r="S64">
+        <v>0</v>
+      </c>
+      <c r="T64">
+        <v>0</v>
+      </c>
+      <c r="U64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>62</v>
+      </c>
+      <c r="B65">
+        <v>63</v>
+      </c>
+      <c r="C65" t="b">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <v>0</v>
+      </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
+      <c r="L65">
+        <v>0</v>
+      </c>
+      <c r="M65">
+        <v>0</v>
+      </c>
+      <c r="N65">
+        <v>0</v>
+      </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65">
+        <v>0</v>
+      </c>
+      <c r="Q65">
+        <v>0</v>
+      </c>
+      <c r="R65">
+        <v>0</v>
+      </c>
+      <c r="S65">
+        <v>0</v>
+      </c>
+      <c r="T65">
+        <v>0</v>
+      </c>
+      <c r="U65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>63</v>
+      </c>
+      <c r="B66">
+        <v>64</v>
+      </c>
+      <c r="C66" t="b">
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <v>0</v>
+      </c>
+      <c r="J66">
+        <v>0</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+      <c r="L66">
+        <v>0</v>
+      </c>
+      <c r="M66">
+        <v>0</v>
+      </c>
+      <c r="N66">
+        <v>0</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>0</v>
+      </c>
+      <c r="Q66">
+        <v>0</v>
+      </c>
+      <c r="R66">
+        <v>0</v>
+      </c>
+      <c r="S66">
+        <v>0</v>
+      </c>
+      <c r="T66">
+        <v>0</v>
+      </c>
+      <c r="U66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>64</v>
+      </c>
+      <c r="B67">
+        <v>65</v>
+      </c>
+      <c r="C67" t="b">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>0</v>
+      </c>
+      <c r="J67">
+        <v>0</v>
+      </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+      <c r="L67">
+        <v>0</v>
+      </c>
+      <c r="M67">
+        <v>0</v>
+      </c>
+      <c r="N67">
+        <v>0</v>
+      </c>
+      <c r="O67">
+        <v>0</v>
+      </c>
+      <c r="P67">
+        <v>0</v>
+      </c>
+      <c r="Q67">
+        <v>0</v>
+      </c>
+      <c r="R67">
+        <v>0</v>
+      </c>
+      <c r="S67">
+        <v>0</v>
+      </c>
+      <c r="T67">
+        <v>0</v>
+      </c>
+      <c r="U67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>65</v>
+      </c>
+      <c r="B68">
+        <v>66</v>
+      </c>
+      <c r="C68" t="b">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+      <c r="J68">
+        <v>0</v>
+      </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
+      <c r="L68">
+        <v>0</v>
+      </c>
+      <c r="M68">
+        <v>0</v>
+      </c>
+      <c r="N68">
+        <v>0</v>
+      </c>
+      <c r="O68">
+        <v>0</v>
+      </c>
+      <c r="P68">
+        <v>0</v>
+      </c>
+      <c r="Q68">
+        <v>0</v>
+      </c>
+      <c r="R68">
+        <v>0</v>
+      </c>
+      <c r="S68">
+        <v>0</v>
+      </c>
+      <c r="T68">
+        <v>0</v>
+      </c>
+      <c r="U68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>66</v>
+      </c>
+      <c r="B69">
+        <v>67</v>
+      </c>
+      <c r="C69" t="b">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>0</v>
+      </c>
+      <c r="J69">
+        <v>0</v>
+      </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
+      <c r="L69">
+        <v>0</v>
+      </c>
+      <c r="M69">
+        <v>0</v>
+      </c>
+      <c r="N69">
+        <v>0</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
+      </c>
+      <c r="P69">
+        <v>0</v>
+      </c>
+      <c r="Q69">
+        <v>0</v>
+      </c>
+      <c r="R69">
+        <v>0</v>
+      </c>
+      <c r="S69">
+        <v>0</v>
+      </c>
+      <c r="T69">
+        <v>0</v>
+      </c>
+      <c r="U69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>67</v>
+      </c>
+      <c r="B70">
+        <v>68</v>
+      </c>
+      <c r="C70" t="b">
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>0</v>
+      </c>
+      <c r="J70">
+        <v>0</v>
+      </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
+      <c r="L70">
+        <v>0</v>
+      </c>
+      <c r="M70">
+        <v>0</v>
+      </c>
+      <c r="N70">
+        <v>0</v>
+      </c>
+      <c r="O70">
+        <v>0</v>
+      </c>
+      <c r="P70">
+        <v>0</v>
+      </c>
+      <c r="Q70">
+        <v>0</v>
+      </c>
+      <c r="R70">
+        <v>0</v>
+      </c>
+      <c r="S70">
+        <v>0</v>
+      </c>
+      <c r="T70">
+        <v>0</v>
+      </c>
+      <c r="U70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>68</v>
+      </c>
+      <c r="B71">
+        <v>69</v>
+      </c>
+      <c r="C71" t="b">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>0</v>
+      </c>
+      <c r="G71">
+        <v>0</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71">
+        <v>0</v>
+      </c>
+      <c r="J71">
+        <v>0</v>
+      </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
+      <c r="L71">
+        <v>0</v>
+      </c>
+      <c r="M71">
+        <v>0</v>
+      </c>
+      <c r="N71">
+        <v>0</v>
+      </c>
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
+        <v>0</v>
+      </c>
+      <c r="Q71">
+        <v>0</v>
+      </c>
+      <c r="R71">
+        <v>0</v>
+      </c>
+      <c r="S71">
+        <v>0</v>
+      </c>
+      <c r="T71">
+        <v>0</v>
+      </c>
+      <c r="U71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>69</v>
+      </c>
+      <c r="B72">
+        <v>70</v>
+      </c>
+      <c r="C72" t="b">
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="G72">
+        <v>0</v>
+      </c>
+      <c r="H72">
+        <v>0</v>
+      </c>
+      <c r="I72">
+        <v>0</v>
+      </c>
+      <c r="J72">
+        <v>0</v>
+      </c>
+      <c r="K72">
+        <v>0</v>
+      </c>
+      <c r="L72">
+        <v>0</v>
+      </c>
+      <c r="M72">
+        <v>0</v>
+      </c>
+      <c r="N72">
+        <v>0</v>
+      </c>
+      <c r="O72">
+        <v>0</v>
+      </c>
+      <c r="P72">
+        <v>0</v>
+      </c>
+      <c r="Q72">
+        <v>0</v>
+      </c>
+      <c r="R72">
+        <v>0</v>
+      </c>
+      <c r="S72">
+        <v>0</v>
+      </c>
+      <c r="T72">
+        <v>0</v>
+      </c>
+      <c r="U72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>70</v>
+      </c>
+      <c r="B73">
+        <v>71</v>
+      </c>
+      <c r="C73" t="b">
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73">
+        <v>0</v>
+      </c>
+      <c r="I73">
+        <v>0</v>
+      </c>
+      <c r="J73">
+        <v>0</v>
+      </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
+      <c r="L73">
+        <v>0</v>
+      </c>
+      <c r="M73">
+        <v>0</v>
+      </c>
+      <c r="N73">
+        <v>0</v>
+      </c>
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
+        <v>0</v>
+      </c>
+      <c r="Q73">
+        <v>0</v>
+      </c>
+      <c r="R73">
+        <v>0</v>
+      </c>
+      <c r="S73">
+        <v>0</v>
+      </c>
+      <c r="T73">
+        <v>0</v>
+      </c>
+      <c r="U73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>71</v>
+      </c>
+      <c r="B74">
+        <v>72</v>
+      </c>
+      <c r="C74" t="b">
+        <v>0</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74">
+        <v>0</v>
+      </c>
+      <c r="I74">
+        <v>0</v>
+      </c>
+      <c r="J74">
+        <v>0</v>
+      </c>
+      <c r="K74">
+        <v>0</v>
+      </c>
+      <c r="L74">
+        <v>0</v>
+      </c>
+      <c r="M74">
+        <v>0</v>
+      </c>
+      <c r="N74">
+        <v>0</v>
+      </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
+        <v>0</v>
+      </c>
+      <c r="Q74">
+        <v>0</v>
+      </c>
+      <c r="R74">
+        <v>0</v>
+      </c>
+      <c r="S74">
+        <v>0</v>
+      </c>
+      <c r="T74">
+        <v>0</v>
+      </c>
+      <c r="U74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>72</v>
+      </c>
+      <c r="B75">
+        <v>73</v>
+      </c>
+      <c r="C75" t="b">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75">
+        <v>0</v>
+      </c>
+      <c r="I75">
+        <v>0</v>
+      </c>
+      <c r="J75">
+        <v>0</v>
+      </c>
+      <c r="K75">
+        <v>0</v>
+      </c>
+      <c r="L75">
+        <v>0</v>
+      </c>
+      <c r="M75">
+        <v>0</v>
+      </c>
+      <c r="N75">
+        <v>0</v>
+      </c>
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
+        <v>0</v>
+      </c>
+      <c r="Q75">
+        <v>0</v>
+      </c>
+      <c r="R75">
+        <v>0</v>
+      </c>
+      <c r="S75">
+        <v>0</v>
+      </c>
+      <c r="T75">
+        <v>0</v>
+      </c>
+      <c r="U75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>73</v>
+      </c>
+      <c r="B76">
+        <v>74</v>
+      </c>
+      <c r="C76" t="b">
+        <v>0</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76">
+        <v>0</v>
+      </c>
+      <c r="I76">
+        <v>0</v>
+      </c>
+      <c r="J76">
+        <v>0</v>
+      </c>
+      <c r="K76">
+        <v>0</v>
+      </c>
+      <c r="L76">
+        <v>0</v>
+      </c>
+      <c r="M76">
+        <v>0</v>
+      </c>
+      <c r="N76">
+        <v>0</v>
+      </c>
+      <c r="O76">
+        <v>0</v>
+      </c>
+      <c r="P76">
+        <v>0</v>
+      </c>
+      <c r="Q76">
+        <v>0</v>
+      </c>
+      <c r="R76">
+        <v>0</v>
+      </c>
+      <c r="S76">
+        <v>0</v>
+      </c>
+      <c r="T76">
+        <v>0</v>
+      </c>
+      <c r="U76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>74</v>
+      </c>
+      <c r="B77">
+        <v>75</v>
+      </c>
+      <c r="C77" t="b">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77">
+        <v>0</v>
+      </c>
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+      <c r="L77">
+        <v>0</v>
+      </c>
+      <c r="M77">
+        <v>0</v>
+      </c>
+      <c r="N77">
+        <v>0</v>
+      </c>
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
+        <v>0</v>
+      </c>
+      <c r="Q77">
+        <v>0</v>
+      </c>
+      <c r="R77">
+        <v>0</v>
+      </c>
+      <c r="S77">
+        <v>0</v>
+      </c>
+      <c r="T77">
+        <v>0</v>
+      </c>
+      <c r="U77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>75</v>
+      </c>
+      <c r="B78">
+        <v>76</v>
+      </c>
+      <c r="C78" t="b">
+        <v>0</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
+        <v>0</v>
+      </c>
+      <c r="I78">
+        <v>0</v>
+      </c>
+      <c r="J78">
+        <v>0</v>
+      </c>
+      <c r="K78">
+        <v>0</v>
+      </c>
+      <c r="L78">
+        <v>0</v>
+      </c>
+      <c r="M78">
+        <v>0</v>
+      </c>
+      <c r="N78">
+        <v>0</v>
+      </c>
+      <c r="O78">
+        <v>0</v>
+      </c>
+      <c r="P78">
+        <v>0</v>
+      </c>
+      <c r="Q78">
+        <v>0</v>
+      </c>
+      <c r="R78">
+        <v>0</v>
+      </c>
+      <c r="S78">
+        <v>0</v>
+      </c>
+      <c r="T78">
+        <v>0</v>
+      </c>
+      <c r="U78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>76</v>
+      </c>
+      <c r="B79">
+        <v>77</v>
+      </c>
+      <c r="C79" t="b">
+        <v>0</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79">
+        <v>0</v>
+      </c>
+      <c r="I79">
+        <v>0</v>
+      </c>
+      <c r="J79">
+        <v>0</v>
+      </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+      <c r="L79">
+        <v>0</v>
+      </c>
+      <c r="M79">
+        <v>0</v>
+      </c>
+      <c r="N79">
+        <v>0</v>
+      </c>
+      <c r="O79">
+        <v>0</v>
+      </c>
+      <c r="P79">
+        <v>0</v>
+      </c>
+      <c r="Q79">
+        <v>0</v>
+      </c>
+      <c r="R79">
+        <v>0</v>
+      </c>
+      <c r="S79">
+        <v>0</v>
+      </c>
+      <c r="T79">
+        <v>0</v>
+      </c>
+      <c r="U79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>77</v>
+      </c>
+      <c r="B80">
+        <v>78</v>
+      </c>
+      <c r="C80" t="b">
+        <v>0</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="G80">
+        <v>0</v>
+      </c>
+      <c r="H80">
+        <v>0</v>
+      </c>
+      <c r="I80">
+        <v>0</v>
+      </c>
+      <c r="J80">
+        <v>0</v>
+      </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80">
+        <v>0</v>
+      </c>
+      <c r="M80">
+        <v>0</v>
+      </c>
+      <c r="N80">
+        <v>0</v>
+      </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80">
+        <v>0</v>
+      </c>
+      <c r="Q80">
+        <v>0</v>
+      </c>
+      <c r="R80">
+        <v>0</v>
+      </c>
+      <c r="S80">
+        <v>0</v>
+      </c>
+      <c r="T80">
+        <v>0</v>
+      </c>
+      <c r="U80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>78</v>
+      </c>
+      <c r="B81">
+        <v>79</v>
+      </c>
+      <c r="C81" t="b">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="G81">
+        <v>0</v>
+      </c>
+      <c r="H81">
+        <v>0</v>
+      </c>
+      <c r="I81">
+        <v>0</v>
+      </c>
+      <c r="J81">
+        <v>0</v>
+      </c>
+      <c r="K81">
+        <v>0</v>
+      </c>
+      <c r="L81">
+        <v>0</v>
+      </c>
+      <c r="M81">
+        <v>0</v>
+      </c>
+      <c r="N81">
+        <v>0</v>
+      </c>
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
+        <v>0</v>
+      </c>
+      <c r="Q81">
+        <v>0</v>
+      </c>
+      <c r="R81">
+        <v>0</v>
+      </c>
+      <c r="S81">
+        <v>0</v>
+      </c>
+      <c r="T81">
+        <v>0</v>
+      </c>
+      <c r="U81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>79</v>
+      </c>
+      <c r="B82">
+        <v>80</v>
+      </c>
+      <c r="C82" t="b">
+        <v>0</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>0</v>
+      </c>
+      <c r="G82">
+        <v>0</v>
+      </c>
+      <c r="H82">
+        <v>0</v>
+      </c>
+      <c r="I82">
+        <v>0</v>
+      </c>
+      <c r="J82">
+        <v>0</v>
+      </c>
+      <c r="K82">
+        <v>0</v>
+      </c>
+      <c r="L82">
+        <v>0</v>
+      </c>
+      <c r="M82">
+        <v>0</v>
+      </c>
+      <c r="N82">
+        <v>0</v>
+      </c>
+      <c r="O82">
+        <v>0</v>
+      </c>
+      <c r="P82">
+        <v>0</v>
+      </c>
+      <c r="Q82">
+        <v>0</v>
+      </c>
+      <c r="R82">
+        <v>0</v>
+      </c>
+      <c r="S82">
+        <v>0</v>
+      </c>
+      <c r="T82">
+        <v>0</v>
+      </c>
+      <c r="U82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>80</v>
+      </c>
+      <c r="B83">
+        <v>81</v>
+      </c>
+      <c r="C83" t="b">
+        <v>0</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>0</v>
+      </c>
+      <c r="J83">
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83">
+        <v>0</v>
+      </c>
+      <c r="M83">
+        <v>0</v>
+      </c>
+      <c r="N83">
+        <v>0</v>
+      </c>
+      <c r="O83">
+        <v>0</v>
+      </c>
+      <c r="P83">
+        <v>0</v>
+      </c>
+      <c r="Q83">
+        <v>0</v>
+      </c>
+      <c r="R83">
+        <v>0</v>
+      </c>
+      <c r="S83">
+        <v>0</v>
+      </c>
+      <c r="T83">
+        <v>0</v>
+      </c>
+      <c r="U83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>81</v>
+      </c>
+      <c r="B84">
+        <v>82</v>
+      </c>
+      <c r="C84" t="b">
+        <v>0</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84">
+        <v>0</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84">
+        <v>0</v>
+      </c>
+      <c r="J84">
+        <v>0</v>
+      </c>
+      <c r="K84">
+        <v>0</v>
+      </c>
+      <c r="L84">
+        <v>0</v>
+      </c>
+      <c r="M84">
+        <v>0</v>
+      </c>
+      <c r="N84">
+        <v>0</v>
+      </c>
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84">
+        <v>0</v>
+      </c>
+      <c r="Q84">
+        <v>0</v>
+      </c>
+      <c r="R84">
+        <v>0</v>
+      </c>
+      <c r="S84">
+        <v>0</v>
+      </c>
+      <c r="T84">
+        <v>0</v>
+      </c>
+      <c r="U84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>82</v>
+      </c>
+      <c r="B85">
+        <v>83</v>
+      </c>
+      <c r="C85" t="b">
+        <v>0</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85">
+        <v>0</v>
+      </c>
+      <c r="J85">
+        <v>0</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85">
+        <v>0</v>
+      </c>
+      <c r="M85">
+        <v>0</v>
+      </c>
+      <c r="N85">
+        <v>0</v>
+      </c>
+      <c r="O85">
+        <v>0</v>
+      </c>
+      <c r="P85">
+        <v>0</v>
+      </c>
+      <c r="Q85">
+        <v>0</v>
+      </c>
+      <c r="R85">
+        <v>0</v>
+      </c>
+      <c r="S85">
+        <v>0</v>
+      </c>
+      <c r="T85">
+        <v>0</v>
+      </c>
+      <c r="U85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>83</v>
+      </c>
+      <c r="B86">
+        <v>84</v>
+      </c>
+      <c r="C86" t="b">
+        <v>0</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86">
+        <v>0</v>
+      </c>
+      <c r="H86">
+        <v>0</v>
+      </c>
+      <c r="I86">
+        <v>0</v>
+      </c>
+      <c r="J86">
+        <v>0</v>
+      </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86">
+        <v>0</v>
+      </c>
+      <c r="M86">
+        <v>0</v>
+      </c>
+      <c r="N86">
+        <v>0</v>
+      </c>
+      <c r="O86">
+        <v>0</v>
+      </c>
+      <c r="P86">
+        <v>0</v>
+      </c>
+      <c r="Q86">
+        <v>0</v>
+      </c>
+      <c r="R86">
+        <v>0</v>
+      </c>
+      <c r="S86">
+        <v>0</v>
+      </c>
+      <c r="T86">
+        <v>0</v>
+      </c>
+      <c r="U86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>84</v>
+      </c>
+      <c r="B87">
+        <v>85</v>
+      </c>
+      <c r="C87" t="b">
+        <v>0</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
+      <c r="I87">
+        <v>0</v>
+      </c>
+      <c r="J87">
+        <v>0</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87">
+        <v>0</v>
+      </c>
+      <c r="M87">
+        <v>0</v>
+      </c>
+      <c r="N87">
+        <v>0</v>
+      </c>
+      <c r="O87">
+        <v>0</v>
+      </c>
+      <c r="P87">
+        <v>0</v>
+      </c>
+      <c r="Q87">
+        <v>0</v>
+      </c>
+      <c r="R87">
+        <v>0</v>
+      </c>
+      <c r="S87">
+        <v>0</v>
+      </c>
+      <c r="T87">
+        <v>0</v>
+      </c>
+      <c r="U87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>85</v>
+      </c>
+      <c r="B88">
+        <v>86</v>
+      </c>
+      <c r="C88" t="b">
+        <v>0</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88">
+        <v>0</v>
+      </c>
+      <c r="H88">
+        <v>0</v>
+      </c>
+      <c r="I88">
+        <v>0</v>
+      </c>
+      <c r="J88">
+        <v>0</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88">
+        <v>0</v>
+      </c>
+      <c r="M88">
+        <v>0</v>
+      </c>
+      <c r="N88">
+        <v>0</v>
+      </c>
+      <c r="O88">
+        <v>0</v>
+      </c>
+      <c r="P88">
+        <v>0</v>
+      </c>
+      <c r="Q88">
+        <v>0</v>
+      </c>
+      <c r="R88">
+        <v>0</v>
+      </c>
+      <c r="S88">
+        <v>0</v>
+      </c>
+      <c r="T88">
+        <v>0</v>
+      </c>
+      <c r="U88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>86</v>
+      </c>
+      <c r="B89">
+        <v>87</v>
+      </c>
+      <c r="C89" t="b">
+        <v>0</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+      <c r="F89">
+        <v>0</v>
+      </c>
+      <c r="G89">
+        <v>0</v>
+      </c>
+      <c r="H89">
+        <v>0</v>
+      </c>
+      <c r="I89">
+        <v>0</v>
+      </c>
+      <c r="J89">
+        <v>0</v>
+      </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
+      <c r="L89">
+        <v>0</v>
+      </c>
+      <c r="M89">
+        <v>0</v>
+      </c>
+      <c r="N89">
+        <v>0</v>
+      </c>
+      <c r="O89">
+        <v>0</v>
+      </c>
+      <c r="P89">
+        <v>0</v>
+      </c>
+      <c r="Q89">
+        <v>0</v>
+      </c>
+      <c r="R89">
+        <v>0</v>
+      </c>
+      <c r="S89">
+        <v>0</v>
+      </c>
+      <c r="T89">
+        <v>0</v>
+      </c>
+      <c r="U89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>87</v>
+      </c>
+      <c r="B90">
+        <v>88</v>
+      </c>
+      <c r="C90" t="b">
+        <v>0</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+      <c r="G90">
+        <v>0</v>
+      </c>
+      <c r="H90">
+        <v>0</v>
+      </c>
+      <c r="I90">
+        <v>0</v>
+      </c>
+      <c r="J90">
+        <v>0</v>
+      </c>
+      <c r="K90">
+        <v>0</v>
+      </c>
+      <c r="L90">
+        <v>0</v>
+      </c>
+      <c r="M90">
+        <v>0</v>
+      </c>
+      <c r="N90">
+        <v>0</v>
+      </c>
+      <c r="O90">
+        <v>0</v>
+      </c>
+      <c r="P90">
+        <v>0</v>
+      </c>
+      <c r="Q90">
+        <v>0</v>
+      </c>
+      <c r="R90">
+        <v>0</v>
+      </c>
+      <c r="S90">
+        <v>0</v>
+      </c>
+      <c r="T90">
+        <v>0</v>
+      </c>
+      <c r="U90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>88</v>
+      </c>
+      <c r="B91">
+        <v>89</v>
+      </c>
+      <c r="C91" t="b">
+        <v>0</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91">
+        <v>0</v>
+      </c>
+      <c r="H91">
+        <v>0</v>
+      </c>
+      <c r="I91">
+        <v>0</v>
+      </c>
+      <c r="J91">
+        <v>0</v>
+      </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
+      <c r="L91">
+        <v>0</v>
+      </c>
+      <c r="M91">
+        <v>0</v>
+      </c>
+      <c r="N91">
+        <v>0</v>
+      </c>
+      <c r="O91">
+        <v>0</v>
+      </c>
+      <c r="P91">
+        <v>0</v>
+      </c>
+      <c r="Q91">
+        <v>0</v>
+      </c>
+      <c r="R91">
+        <v>0</v>
+      </c>
+      <c r="S91">
+        <v>0</v>
+      </c>
+      <c r="T91">
+        <v>0</v>
+      </c>
+      <c r="U91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>89</v>
+      </c>
+      <c r="B92">
+        <v>90</v>
+      </c>
+      <c r="C92" t="b">
+        <v>0</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>0</v>
+      </c>
+      <c r="G92">
+        <v>0</v>
+      </c>
+      <c r="H92">
+        <v>0</v>
+      </c>
+      <c r="I92">
+        <v>0</v>
+      </c>
+      <c r="J92">
+        <v>0</v>
+      </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
+      <c r="L92">
+        <v>0</v>
+      </c>
+      <c r="M92">
+        <v>0</v>
+      </c>
+      <c r="N92">
+        <v>0</v>
+      </c>
+      <c r="O92">
+        <v>0</v>
+      </c>
+      <c r="P92">
+        <v>0</v>
+      </c>
+      <c r="Q92">
+        <v>0</v>
+      </c>
+      <c r="R92">
+        <v>0</v>
+      </c>
+      <c r="S92">
+        <v>0</v>
+      </c>
+      <c r="T92">
+        <v>0</v>
+      </c>
+      <c r="U92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>90</v>
+      </c>
+      <c r="B93">
+        <v>91</v>
+      </c>
+      <c r="C93" t="b">
+        <v>0</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+      <c r="G93">
+        <v>0</v>
+      </c>
+      <c r="H93">
+        <v>0</v>
+      </c>
+      <c r="I93">
+        <v>-1</v>
+      </c>
+      <c r="J93">
+        <v>0</v>
+      </c>
+      <c r="K93">
+        <v>0</v>
+      </c>
+      <c r="L93">
+        <v>0</v>
+      </c>
+      <c r="M93">
+        <v>0</v>
+      </c>
+      <c r="N93">
+        <v>0</v>
+      </c>
+      <c r="O93">
+        <v>0</v>
+      </c>
+      <c r="P93">
+        <v>0</v>
+      </c>
+      <c r="Q93">
+        <v>0</v>
+      </c>
+      <c r="R93">
+        <v>0</v>
+      </c>
+      <c r="S93">
+        <v>0</v>
+      </c>
+      <c r="T93">
+        <v>0</v>
+      </c>
+      <c r="U93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>91</v>
+      </c>
+      <c r="B94">
+        <v>92</v>
+      </c>
+      <c r="C94" t="b">
+        <v>0</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="G94">
+        <v>0</v>
+      </c>
+      <c r="H94">
+        <v>0</v>
+      </c>
+      <c r="I94">
+        <v>-1</v>
+      </c>
+      <c r="J94">
+        <v>0</v>
+      </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
+      <c r="L94">
+        <v>0</v>
+      </c>
+      <c r="M94">
+        <v>0</v>
+      </c>
+      <c r="N94">
+        <v>0</v>
+      </c>
+      <c r="O94">
+        <v>0</v>
+      </c>
+      <c r="P94">
+        <v>0</v>
+      </c>
+      <c r="Q94">
+        <v>0</v>
+      </c>
+      <c r="R94">
+        <v>0</v>
+      </c>
+      <c r="S94">
+        <v>0</v>
+      </c>
+      <c r="T94">
+        <v>0</v>
+      </c>
+      <c r="U94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>92</v>
+      </c>
+      <c r="B95">
+        <v>93</v>
+      </c>
+      <c r="C95" t="b">
+        <v>0</v>
+      </c>
+      <c r="D95">
+        <v>0</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="G95">
+        <v>0</v>
+      </c>
+      <c r="H95">
+        <v>0</v>
+      </c>
+      <c r="I95">
+        <v>-1</v>
+      </c>
+      <c r="J95">
+        <v>0</v>
+      </c>
+      <c r="K95">
+        <v>0</v>
+      </c>
+      <c r="L95">
+        <v>0</v>
+      </c>
+      <c r="M95">
+        <v>0</v>
+      </c>
+      <c r="N95">
+        <v>0</v>
+      </c>
+      <c r="O95">
+        <v>0</v>
+      </c>
+      <c r="P95">
+        <v>0</v>
+      </c>
+      <c r="Q95">
+        <v>0</v>
+      </c>
+      <c r="R95">
+        <v>0</v>
+      </c>
+      <c r="S95">
+        <v>0</v>
+      </c>
+      <c r="T95">
+        <v>0</v>
+      </c>
+      <c r="U95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>93</v>
+      </c>
+      <c r="B96">
+        <v>94</v>
+      </c>
+      <c r="C96" t="b">
+        <v>0</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96">
+        <v>0</v>
+      </c>
+      <c r="H96">
+        <v>0</v>
+      </c>
+      <c r="I96">
+        <v>-1</v>
+      </c>
+      <c r="J96">
+        <v>0</v>
+      </c>
+      <c r="K96">
+        <v>0</v>
+      </c>
+      <c r="L96">
+        <v>0</v>
+      </c>
+      <c r="M96">
+        <v>0</v>
+      </c>
+      <c r="N96">
+        <v>0</v>
+      </c>
+      <c r="O96">
+        <v>0</v>
+      </c>
+      <c r="P96">
+        <v>0</v>
+      </c>
+      <c r="Q96">
+        <v>0</v>
+      </c>
+      <c r="R96">
+        <v>0</v>
+      </c>
+      <c r="S96">
+        <v>0</v>
+      </c>
+      <c r="T96">
+        <v>0</v>
+      </c>
+      <c r="U96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>94</v>
+      </c>
+      <c r="B97">
+        <v>95</v>
+      </c>
+      <c r="C97" t="b">
+        <v>0</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97">
+        <v>0</v>
+      </c>
+      <c r="H97">
+        <v>0</v>
+      </c>
+      <c r="I97">
+        <v>-1</v>
+      </c>
+      <c r="J97">
+        <v>0</v>
+      </c>
+      <c r="K97">
+        <v>0</v>
+      </c>
+      <c r="L97">
+        <v>0</v>
+      </c>
+      <c r="M97">
+        <v>0</v>
+      </c>
+      <c r="N97">
+        <v>0</v>
+      </c>
+      <c r="O97">
+        <v>0</v>
+      </c>
+      <c r="P97">
+        <v>0</v>
+      </c>
+      <c r="Q97">
+        <v>0</v>
+      </c>
+      <c r="R97">
+        <v>0</v>
+      </c>
+      <c r="S97">
+        <v>0</v>
+      </c>
+      <c r="T97">
+        <v>0</v>
+      </c>
+      <c r="U97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>95</v>
+      </c>
+      <c r="B98">
+        <v>96</v>
+      </c>
+      <c r="C98" t="b">
+        <v>0</v>
+      </c>
+      <c r="D98">
+        <v>0</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98">
+        <v>0</v>
+      </c>
+      <c r="H98">
+        <v>0</v>
+      </c>
+      <c r="I98">
+        <v>-1</v>
+      </c>
+      <c r="J98">
+        <v>0</v>
+      </c>
+      <c r="K98">
+        <v>0</v>
+      </c>
+      <c r="L98">
+        <v>0</v>
+      </c>
+      <c r="M98">
+        <v>0</v>
+      </c>
+      <c r="N98">
+        <v>0</v>
+      </c>
+      <c r="O98">
+        <v>0</v>
+      </c>
+      <c r="P98">
+        <v>0</v>
+      </c>
+      <c r="Q98">
+        <v>0</v>
+      </c>
+      <c r="R98">
+        <v>0</v>
+      </c>
+      <c r="S98">
+        <v>0</v>
+      </c>
+      <c r="T98">
+        <v>0</v>
+      </c>
+      <c r="U98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>96</v>
+      </c>
+      <c r="B99">
+        <v>97</v>
+      </c>
+      <c r="C99" t="b">
+        <v>0</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="G99">
+        <v>0</v>
+      </c>
+      <c r="H99">
+        <v>0</v>
+      </c>
+      <c r="I99">
+        <v>-1</v>
+      </c>
+      <c r="J99">
+        <v>0</v>
+      </c>
+      <c r="K99">
+        <v>0</v>
+      </c>
+      <c r="L99">
+        <v>0</v>
+      </c>
+      <c r="M99">
+        <v>0</v>
+      </c>
+      <c r="N99">
+        <v>0</v>
+      </c>
+      <c r="O99">
+        <v>0</v>
+      </c>
+      <c r="P99">
+        <v>0</v>
+      </c>
+      <c r="Q99">
+        <v>0</v>
+      </c>
+      <c r="R99">
+        <v>0</v>
+      </c>
+      <c r="S99">
+        <v>0</v>
+      </c>
+      <c r="T99">
+        <v>0</v>
+      </c>
+      <c r="U99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>97</v>
+      </c>
+      <c r="B100">
+        <v>98</v>
+      </c>
+      <c r="C100" t="b">
+        <v>0</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>0</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+      <c r="G100">
+        <v>0</v>
+      </c>
+      <c r="H100">
+        <v>0</v>
+      </c>
+      <c r="I100">
+        <v>-1</v>
+      </c>
+      <c r="J100">
+        <v>0</v>
+      </c>
+      <c r="K100">
+        <v>0</v>
+      </c>
+      <c r="L100">
+        <v>0</v>
+      </c>
+      <c r="M100">
+        <v>0</v>
+      </c>
+      <c r="N100">
+        <v>0</v>
+      </c>
+      <c r="O100">
+        <v>0</v>
+      </c>
+      <c r="P100">
+        <v>0</v>
+      </c>
+      <c r="Q100">
+        <v>0</v>
+      </c>
+      <c r="R100">
+        <v>0</v>
+      </c>
+      <c r="S100">
+        <v>0</v>
+      </c>
+      <c r="T100">
+        <v>0</v>
+      </c>
+      <c r="U100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>98</v>
+      </c>
+      <c r="B101">
+        <v>99</v>
+      </c>
+      <c r="C101" t="b">
+        <v>0</v>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>0</v>
+      </c>
+      <c r="G101">
+        <v>0</v>
+      </c>
+      <c r="H101">
+        <v>0</v>
+      </c>
+      <c r="I101">
+        <v>-1</v>
+      </c>
+      <c r="J101">
+        <v>0</v>
+      </c>
+      <c r="K101">
+        <v>0</v>
+      </c>
+      <c r="L101">
+        <v>0</v>
+      </c>
+      <c r="M101">
+        <v>0</v>
+      </c>
+      <c r="N101">
+        <v>0</v>
+      </c>
+      <c r="O101">
+        <v>0</v>
+      </c>
+      <c r="P101">
+        <v>0</v>
+      </c>
+      <c r="Q101">
+        <v>0</v>
+      </c>
+      <c r="R101">
+        <v>0</v>
+      </c>
+      <c r="S101">
+        <v>0</v>
+      </c>
+      <c r="T101">
+        <v>0</v>
+      </c>
+      <c r="U101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>99</v>
+      </c>
+      <c r="B102">
+        <v>100</v>
+      </c>
+      <c r="C102" t="b">
+        <v>0</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>0</v>
+      </c>
+      <c r="G102">
+        <v>0</v>
+      </c>
+      <c r="H102">
+        <v>0</v>
+      </c>
+      <c r="I102">
+        <v>-1</v>
+      </c>
+      <c r="J102">
+        <v>0</v>
+      </c>
+      <c r="K102">
+        <v>0</v>
+      </c>
+      <c r="L102">
+        <v>0</v>
+      </c>
+      <c r="M102">
+        <v>0</v>
+      </c>
+      <c r="N102">
+        <v>0</v>
+      </c>
+      <c r="O102">
+        <v>0</v>
+      </c>
+      <c r="P102">
+        <v>0</v>
+      </c>
+      <c r="Q102">
+        <v>0</v>
+      </c>
+      <c r="R102">
+        <v>0</v>
+      </c>
+      <c r="S102">
+        <v>0</v>
+      </c>
+      <c r="T102">
+        <v>0</v>
+      </c>
+      <c r="U102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>100</v>
+      </c>
+      <c r="B103">
+        <v>101</v>
+      </c>
+      <c r="C103" t="b">
+        <v>0</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+      <c r="G103">
+        <v>0</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+      <c r="I103">
+        <v>-1</v>
+      </c>
+      <c r="J103">
+        <v>0</v>
+      </c>
+      <c r="K103">
+        <v>0</v>
+      </c>
+      <c r="L103">
+        <v>0</v>
+      </c>
+      <c r="M103">
+        <v>0</v>
+      </c>
+      <c r="N103">
+        <v>0</v>
+      </c>
+      <c r="O103">
+        <v>0</v>
+      </c>
+      <c r="P103">
+        <v>0</v>
+      </c>
+      <c r="Q103">
+        <v>0</v>
+      </c>
+      <c r="R103">
+        <v>0</v>
+      </c>
+      <c r="S103">
+        <v>0</v>
+      </c>
+      <c r="T103">
+        <v>0</v>
+      </c>
+      <c r="U103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>101</v>
+      </c>
+      <c r="B104">
+        <v>102</v>
+      </c>
+      <c r="C104" t="b">
+        <v>0</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>0</v>
+      </c>
+      <c r="F104">
+        <v>0</v>
+      </c>
+      <c r="G104">
+        <v>0</v>
+      </c>
+      <c r="H104">
+        <v>0</v>
+      </c>
+      <c r="I104">
+        <v>-1</v>
+      </c>
+      <c r="J104">
+        <v>0</v>
+      </c>
+      <c r="K104">
+        <v>0</v>
+      </c>
+      <c r="L104">
+        <v>0</v>
+      </c>
+      <c r="M104">
+        <v>0</v>
+      </c>
+      <c r="N104">
+        <v>0</v>
+      </c>
+      <c r="O104">
+        <v>0</v>
+      </c>
+      <c r="P104">
+        <v>0</v>
+      </c>
+      <c r="Q104">
+        <v>0</v>
+      </c>
+      <c r="R104">
+        <v>0</v>
+      </c>
+      <c r="S104">
+        <v>0</v>
+      </c>
+      <c r="T104">
+        <v>0</v>
+      </c>
+      <c r="U104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>102</v>
+      </c>
+      <c r="B105">
+        <v>103</v>
+      </c>
+      <c r="C105" t="b">
+        <v>0</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>0</v>
+      </c>
+      <c r="G105">
+        <v>0</v>
+      </c>
+      <c r="H105">
+        <v>0</v>
+      </c>
+      <c r="I105">
+        <v>-1</v>
+      </c>
+      <c r="J105">
+        <v>0</v>
+      </c>
+      <c r="K105">
+        <v>0</v>
+      </c>
+      <c r="L105">
+        <v>0</v>
+      </c>
+      <c r="M105">
+        <v>0</v>
+      </c>
+      <c r="N105">
+        <v>0</v>
+      </c>
+      <c r="O105">
+        <v>0</v>
+      </c>
+      <c r="P105">
+        <v>0</v>
+      </c>
+      <c r="Q105">
+        <v>0</v>
+      </c>
+      <c r="R105">
+        <v>0</v>
+      </c>
+      <c r="S105">
+        <v>0</v>
+      </c>
+      <c r="T105">
+        <v>0</v>
+      </c>
+      <c r="U105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>103</v>
+      </c>
+      <c r="B106">
+        <v>104</v>
+      </c>
+      <c r="C106" t="b">
+        <v>0</v>
+      </c>
+      <c r="D106">
+        <v>0</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>0</v>
+      </c>
+      <c r="G106">
+        <v>0</v>
+      </c>
+      <c r="H106">
+        <v>0</v>
+      </c>
+      <c r="I106">
+        <v>-1</v>
+      </c>
+      <c r="J106">
+        <v>0</v>
+      </c>
+      <c r="K106">
+        <v>0</v>
+      </c>
+      <c r="L106">
+        <v>0</v>
+      </c>
+      <c r="M106">
+        <v>0</v>
+      </c>
+      <c r="N106">
+        <v>0</v>
+      </c>
+      <c r="O106">
+        <v>0</v>
+      </c>
+      <c r="P106">
+        <v>0</v>
+      </c>
+      <c r="Q106">
+        <v>0</v>
+      </c>
+      <c r="R106">
+        <v>0</v>
+      </c>
+      <c r="S106">
+        <v>0</v>
+      </c>
+      <c r="T106">
+        <v>0</v>
+      </c>
+      <c r="U106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>104</v>
+      </c>
+      <c r="B107">
+        <v>105</v>
+      </c>
+      <c r="C107" t="b">
+        <v>0</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>0</v>
+      </c>
+      <c r="G107">
+        <v>0</v>
+      </c>
+      <c r="H107">
+        <v>0</v>
+      </c>
+      <c r="I107">
+        <v>-1</v>
+      </c>
+      <c r="J107">
+        <v>0</v>
+      </c>
+      <c r="K107">
+        <v>0</v>
+      </c>
+      <c r="L107">
+        <v>0</v>
+      </c>
+      <c r="M107">
+        <v>0</v>
+      </c>
+      <c r="N107">
+        <v>0</v>
+      </c>
+      <c r="O107">
+        <v>0</v>
+      </c>
+      <c r="P107">
+        <v>0</v>
+      </c>
+      <c r="Q107">
+        <v>0</v>
+      </c>
+      <c r="R107">
+        <v>0</v>
+      </c>
+      <c r="S107">
+        <v>0</v>
+      </c>
+      <c r="T107">
+        <v>0</v>
+      </c>
+      <c r="U107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>105</v>
+      </c>
+      <c r="B108">
+        <v>106</v>
+      </c>
+      <c r="C108" t="b">
+        <v>0</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108">
+        <v>0</v>
+      </c>
+      <c r="F108">
+        <v>0</v>
+      </c>
+      <c r="G108">
+        <v>0</v>
+      </c>
+      <c r="H108">
+        <v>0</v>
+      </c>
+      <c r="I108">
+        <v>-1</v>
+      </c>
+      <c r="J108">
+        <v>0</v>
+      </c>
+      <c r="K108">
+        <v>0</v>
+      </c>
+      <c r="L108">
+        <v>0</v>
+      </c>
+      <c r="M108">
+        <v>0</v>
+      </c>
+      <c r="N108">
+        <v>0</v>
+      </c>
+      <c r="O108">
+        <v>0</v>
+      </c>
+      <c r="P108">
+        <v>0</v>
+      </c>
+      <c r="Q108">
+        <v>0</v>
+      </c>
+      <c r="R108">
+        <v>0</v>
+      </c>
+      <c r="S108">
+        <v>0</v>
+      </c>
+      <c r="T108">
+        <v>0</v>
+      </c>
+      <c r="U108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>106</v>
+      </c>
+      <c r="B109">
+        <v>107</v>
+      </c>
+      <c r="C109" t="b">
+        <v>0</v>
+      </c>
+      <c r="D109">
+        <v>0</v>
+      </c>
+      <c r="E109">
+        <v>0</v>
+      </c>
+      <c r="F109">
+        <v>0</v>
+      </c>
+      <c r="G109">
+        <v>0</v>
+      </c>
+      <c r="H109">
+        <v>0</v>
+      </c>
+      <c r="I109">
+        <v>-1</v>
+      </c>
+      <c r="J109">
+        <v>0</v>
+      </c>
+      <c r="K109">
+        <v>0</v>
+      </c>
+      <c r="L109">
+        <v>0</v>
+      </c>
+      <c r="M109">
+        <v>0</v>
+      </c>
+      <c r="N109">
+        <v>0</v>
+      </c>
+      <c r="O109">
+        <v>0</v>
+      </c>
+      <c r="P109">
+        <v>0</v>
+      </c>
+      <c r="Q109">
+        <v>0</v>
+      </c>
+      <c r="R109">
+        <v>0</v>
+      </c>
+      <c r="S109">
+        <v>0</v>
+      </c>
+      <c r="T109">
+        <v>0</v>
+      </c>
+      <c r="U109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>107</v>
+      </c>
+      <c r="B110">
+        <v>108</v>
+      </c>
+      <c r="C110" t="b">
+        <v>0</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110">
+        <v>0</v>
+      </c>
+      <c r="F110">
+        <v>0</v>
+      </c>
+      <c r="G110">
+        <v>0</v>
+      </c>
+      <c r="H110">
+        <v>0</v>
+      </c>
+      <c r="I110">
+        <v>-1</v>
+      </c>
+      <c r="J110">
+        <v>0</v>
+      </c>
+      <c r="K110">
+        <v>0</v>
+      </c>
+      <c r="L110">
+        <v>0</v>
+      </c>
+      <c r="M110">
+        <v>0</v>
+      </c>
+      <c r="N110">
+        <v>0</v>
+      </c>
+      <c r="O110">
+        <v>0</v>
+      </c>
+      <c r="P110">
+        <v>0</v>
+      </c>
+      <c r="Q110">
+        <v>0</v>
+      </c>
+      <c r="R110">
+        <v>0</v>
+      </c>
+      <c r="S110">
+        <v>0</v>
+      </c>
+      <c r="T110">
+        <v>0</v>
+      </c>
+      <c r="U110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>108</v>
+      </c>
+      <c r="B111">
+        <v>109</v>
+      </c>
+      <c r="C111" t="b">
+        <v>0</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111">
+        <v>0</v>
+      </c>
+      <c r="F111">
+        <v>0</v>
+      </c>
+      <c r="G111">
+        <v>0</v>
+      </c>
+      <c r="H111">
+        <v>0</v>
+      </c>
+      <c r="I111">
+        <v>-1</v>
+      </c>
+      <c r="J111">
+        <v>0</v>
+      </c>
+      <c r="K111">
+        <v>0</v>
+      </c>
+      <c r="L111">
+        <v>0</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111">
+        <v>0</v>
+      </c>
+      <c r="O111">
+        <v>0</v>
+      </c>
+      <c r="P111">
+        <v>0</v>
+      </c>
+      <c r="Q111">
+        <v>0</v>
+      </c>
+      <c r="R111">
+        <v>0</v>
+      </c>
+      <c r="S111">
+        <v>0</v>
+      </c>
+      <c r="T111">
+        <v>0</v>
+      </c>
+      <c r="U111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>109</v>
+      </c>
+      <c r="B112">
+        <v>110</v>
+      </c>
+      <c r="C112" t="b">
+        <v>0</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>0</v>
+      </c>
+      <c r="G112">
+        <v>0</v>
+      </c>
+      <c r="H112">
+        <v>0</v>
+      </c>
+      <c r="I112">
+        <v>-1</v>
+      </c>
+      <c r="J112">
+        <v>0</v>
+      </c>
+      <c r="K112">
+        <v>0</v>
+      </c>
+      <c r="L112">
+        <v>0</v>
+      </c>
+      <c r="M112">
+        <v>0</v>
+      </c>
+      <c r="N112">
+        <v>0</v>
+      </c>
+      <c r="O112">
+        <v>0</v>
+      </c>
+      <c r="P112">
+        <v>0</v>
+      </c>
+      <c r="Q112">
+        <v>0</v>
+      </c>
+      <c r="R112">
+        <v>0</v>
+      </c>
+      <c r="S112">
+        <v>0</v>
+      </c>
+      <c r="T112">
+        <v>0</v>
+      </c>
+      <c r="U112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>110</v>
+      </c>
+      <c r="B113">
+        <v>111</v>
+      </c>
+      <c r="C113" t="b">
+        <v>0</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>0</v>
+      </c>
+      <c r="G113">
+        <v>0</v>
+      </c>
+      <c r="H113">
+        <v>0</v>
+      </c>
+      <c r="I113">
+        <v>-1</v>
+      </c>
+      <c r="J113">
+        <v>0</v>
+      </c>
+      <c r="K113">
+        <v>0</v>
+      </c>
+      <c r="L113">
+        <v>0</v>
+      </c>
+      <c r="M113">
+        <v>0</v>
+      </c>
+      <c r="N113">
+        <v>0</v>
+      </c>
+      <c r="O113">
+        <v>0</v>
+      </c>
+      <c r="P113">
+        <v>0</v>
+      </c>
+      <c r="Q113">
+        <v>0</v>
+      </c>
+      <c r="R113">
+        <v>0</v>
+      </c>
+      <c r="S113">
+        <v>0</v>
+      </c>
+      <c r="T113">
+        <v>0</v>
+      </c>
+      <c r="U113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>111</v>
+      </c>
+      <c r="B114">
+        <v>112</v>
+      </c>
+      <c r="C114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D114">
+        <v>0</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>0</v>
+      </c>
+      <c r="G114">
+        <v>0</v>
+      </c>
+      <c r="H114">
+        <v>0</v>
+      </c>
+      <c r="I114">
+        <v>-1</v>
+      </c>
+      <c r="J114">
+        <v>0</v>
+      </c>
+      <c r="K114">
+        <v>0</v>
+      </c>
+      <c r="L114">
+        <v>0</v>
+      </c>
+      <c r="M114">
+        <v>0</v>
+      </c>
+      <c r="N114">
+        <v>0</v>
+      </c>
+      <c r="O114">
+        <v>0</v>
+      </c>
+      <c r="P114">
+        <v>0</v>
+      </c>
+      <c r="Q114">
+        <v>0</v>
+      </c>
+      <c r="R114">
+        <v>0</v>
+      </c>
+      <c r="S114">
+        <v>0</v>
+      </c>
+      <c r="T114">
+        <v>0</v>
+      </c>
+      <c r="U114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>112</v>
+      </c>
+      <c r="B115">
+        <v>113</v>
+      </c>
+      <c r="C115" t="b">
+        <v>0</v>
+      </c>
+      <c r="D115">
+        <v>0</v>
+      </c>
+      <c r="E115">
+        <v>0</v>
+      </c>
+      <c r="F115">
+        <v>0</v>
+      </c>
+      <c r="G115">
+        <v>0</v>
+      </c>
+      <c r="H115">
+        <v>0</v>
+      </c>
+      <c r="I115">
+        <v>-1</v>
+      </c>
+      <c r="J115">
+        <v>0</v>
+      </c>
+      <c r="K115">
+        <v>0</v>
+      </c>
+      <c r="L115">
+        <v>0</v>
+      </c>
+      <c r="M115">
+        <v>0</v>
+      </c>
+      <c r="N115">
+        <v>0</v>
+      </c>
+      <c r="O115">
+        <v>0</v>
+      </c>
+      <c r="P115">
+        <v>0</v>
+      </c>
+      <c r="Q115">
+        <v>0</v>
+      </c>
+      <c r="R115">
+        <v>0</v>
+      </c>
+      <c r="S115">
+        <v>0</v>
+      </c>
+      <c r="T115">
+        <v>0</v>
+      </c>
+      <c r="U115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>113</v>
+      </c>
+      <c r="B116">
+        <v>114</v>
+      </c>
+      <c r="C116" t="b">
+        <v>0</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116">
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <v>0</v>
+      </c>
+      <c r="H116">
+        <v>0</v>
+      </c>
+      <c r="I116">
+        <v>-1</v>
+      </c>
+      <c r="J116">
+        <v>0</v>
+      </c>
+      <c r="K116">
+        <v>0</v>
+      </c>
+      <c r="L116">
+        <v>0</v>
+      </c>
+      <c r="M116">
+        <v>0</v>
+      </c>
+      <c r="N116">
+        <v>0</v>
+      </c>
+      <c r="O116">
+        <v>0</v>
+      </c>
+      <c r="P116">
+        <v>0</v>
+      </c>
+      <c r="Q116">
+        <v>0</v>
+      </c>
+      <c r="R116">
+        <v>0</v>
+      </c>
+      <c r="S116">
+        <v>0</v>
+      </c>
+      <c r="T116">
+        <v>0</v>
+      </c>
+      <c r="U116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>114</v>
+      </c>
+      <c r="B117">
+        <v>115</v>
+      </c>
+      <c r="C117" t="b">
+        <v>0</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <v>0</v>
+      </c>
+      <c r="H117">
+        <v>0</v>
+      </c>
+      <c r="I117">
+        <v>-1</v>
+      </c>
+      <c r="J117">
+        <v>0</v>
+      </c>
+      <c r="K117">
+        <v>0</v>
+      </c>
+      <c r="L117">
+        <v>0</v>
+      </c>
+      <c r="M117">
+        <v>0</v>
+      </c>
+      <c r="N117">
+        <v>0</v>
+      </c>
+      <c r="O117">
+        <v>0</v>
+      </c>
+      <c r="P117">
+        <v>0</v>
+      </c>
+      <c r="Q117">
+        <v>0</v>
+      </c>
+      <c r="R117">
+        <v>0</v>
+      </c>
+      <c r="S117">
+        <v>0</v>
+      </c>
+      <c r="T117">
+        <v>0</v>
+      </c>
+      <c r="U117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>115</v>
+      </c>
+      <c r="B118">
+        <v>116</v>
+      </c>
+      <c r="C118" t="b">
+        <v>0</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <v>0</v>
+      </c>
+      <c r="H118">
+        <v>0</v>
+      </c>
+      <c r="I118">
+        <v>-1</v>
+      </c>
+      <c r="J118">
+        <v>0</v>
+      </c>
+      <c r="K118">
+        <v>0</v>
+      </c>
+      <c r="L118">
+        <v>0</v>
+      </c>
+      <c r="M118">
+        <v>0</v>
+      </c>
+      <c r="N118">
+        <v>0</v>
+      </c>
+      <c r="O118">
+        <v>0</v>
+      </c>
+      <c r="P118">
+        <v>0</v>
+      </c>
+      <c r="Q118">
+        <v>0</v>
+      </c>
+      <c r="R118">
+        <v>0</v>
+      </c>
+      <c r="S118">
+        <v>0</v>
+      </c>
+      <c r="T118">
+        <v>0</v>
+      </c>
+      <c r="U118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>116</v>
+      </c>
+      <c r="B119">
+        <v>117</v>
+      </c>
+      <c r="C119" t="b">
+        <v>0</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119">
+        <v>0</v>
+      </c>
+      <c r="F119">
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <v>0</v>
+      </c>
+      <c r="H119">
+        <v>0</v>
+      </c>
+      <c r="I119">
+        <v>-1</v>
+      </c>
+      <c r="J119">
+        <v>0</v>
+      </c>
+      <c r="K119">
+        <v>0</v>
+      </c>
+      <c r="L119">
+        <v>0</v>
+      </c>
+      <c r="M119">
+        <v>0</v>
+      </c>
+      <c r="N119">
+        <v>0</v>
+      </c>
+      <c r="O119">
+        <v>0</v>
+      </c>
+      <c r="P119">
+        <v>0</v>
+      </c>
+      <c r="Q119">
+        <v>0</v>
+      </c>
+      <c r="R119">
+        <v>0</v>
+      </c>
+      <c r="S119">
+        <v>0</v>
+      </c>
+      <c r="T119">
+        <v>0</v>
+      </c>
+      <c r="U119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>117</v>
+      </c>
+      <c r="B120">
+        <v>118</v>
+      </c>
+      <c r="C120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>0</v>
+      </c>
+      <c r="G120">
+        <v>0</v>
+      </c>
+      <c r="H120">
+        <v>0</v>
+      </c>
+      <c r="I120">
+        <v>-1</v>
+      </c>
+      <c r="J120">
+        <v>0</v>
+      </c>
+      <c r="K120">
+        <v>0</v>
+      </c>
+      <c r="L120">
+        <v>0</v>
+      </c>
+      <c r="M120">
+        <v>0</v>
+      </c>
+      <c r="N120">
+        <v>0</v>
+      </c>
+      <c r="O120">
+        <v>0</v>
+      </c>
+      <c r="P120">
+        <v>0</v>
+      </c>
+      <c r="Q120">
+        <v>0</v>
+      </c>
+      <c r="R120">
+        <v>0</v>
+      </c>
+      <c r="S120">
+        <v>0</v>
+      </c>
+      <c r="T120">
+        <v>0</v>
+      </c>
+      <c r="U120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>118</v>
+      </c>
+      <c r="B121">
+        <v>119</v>
+      </c>
+      <c r="C121" t="b">
+        <v>0</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121">
+        <v>0</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+      <c r="G121">
+        <v>0</v>
+      </c>
+      <c r="H121">
+        <v>0</v>
+      </c>
+      <c r="I121">
+        <v>-1</v>
+      </c>
+      <c r="J121">
+        <v>0</v>
+      </c>
+      <c r="K121">
+        <v>0</v>
+      </c>
+      <c r="L121">
+        <v>0</v>
+      </c>
+      <c r="M121">
+        <v>0</v>
+      </c>
+      <c r="N121">
+        <v>0</v>
+      </c>
+      <c r="O121">
+        <v>0</v>
+      </c>
+      <c r="P121">
+        <v>0</v>
+      </c>
+      <c r="Q121">
+        <v>0</v>
+      </c>
+      <c r="R121">
+        <v>0</v>
+      </c>
+      <c r="S121">
+        <v>0</v>
+      </c>
+      <c r="T121">
+        <v>0</v>
+      </c>
+      <c r="U121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>119</v>
+      </c>
+      <c r="B122">
+        <v>120</v>
+      </c>
+      <c r="C122" t="b">
+        <v>0</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122">
+        <v>0</v>
+      </c>
+      <c r="F122">
+        <v>0</v>
+      </c>
+      <c r="G122">
+        <v>0</v>
+      </c>
+      <c r="H122">
+        <v>0</v>
+      </c>
+      <c r="I122">
+        <v>-1</v>
+      </c>
+      <c r="J122">
+        <v>0</v>
+      </c>
+      <c r="K122">
+        <v>0</v>
+      </c>
+      <c r="L122">
+        <v>0</v>
+      </c>
+      <c r="M122">
+        <v>0</v>
+      </c>
+      <c r="N122">
+        <v>0</v>
+      </c>
+      <c r="O122">
+        <v>0</v>
+      </c>
+      <c r="P122">
+        <v>0</v>
+      </c>
+      <c r="Q122">
+        <v>0</v>
+      </c>
+      <c r="R122">
+        <v>0</v>
+      </c>
+      <c r="S122">
+        <v>0</v>
+      </c>
+      <c r="T122">
+        <v>0</v>
+      </c>
+      <c r="U122">
         <v>0</v>
       </c>
     </row>
@@ -24235,7 +28135,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -28275,7 +32175,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -32316,7 +36216,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -36356,7 +40256,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -40396,7 +44296,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -44436,7 +48336,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -48476,7 +52376,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="B2">
         <v>0</v>

</xml_diff>